<commit_message>
Finished: En verimli Model oluşturuldu. Notlar kısmında karşılaştırmaları ve grafikleri mevcuttur. En son eklenen Best-v7-Model projenin main kısmındadır.
</commit_message>
<xml_diff>
--- a/Notlar/Sonuçlar-v2.xlsx
+++ b/Notlar/Sonuçlar-v2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dunda\OneDrive\Masaüstü\Depression-Analysis-DL\Notlar\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dunda\OneDrive\Masaüstü\Depresyon Analizi\Depression-Analysis-DL\Notlar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71B8343B-3843-4D7C-9A37-72341AD16EB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79F57A5E-D1CD-469C-9BB7-21F352A4C8BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="90">
   <si>
     <t>1/1 [==============================] - 2s 2s/step</t>
   </si>
@@ -96,7 +96,205 @@
     <t>Depression Probability: 0.0563</t>
   </si>
   <si>
-    <t>Current-Model --- 09.12.2024 - 12.45</t>
+    <t>Best-v1-Model   09.12.2024 - 12.45</t>
+  </si>
+  <si>
+    <t>Best-v2-Model  09.12.2024 - 15.53</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.7748</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0588</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.9552</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0143</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.9133</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0585</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.9387</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0064</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.4552</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0319</t>
+  </si>
+  <si>
+    <t>Best-v3-Model  09.12.2024 - 18.11</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0284</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.7786</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0309</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.9273</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0083</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.8623</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.1045</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.9190</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0133</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.7859</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0557</t>
+  </si>
+  <si>
+    <t>Best-v4-Model  09.12.2024 - 19.44</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.8630</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0273</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.9202</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0178</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.8805</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.1381</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.9322</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0458</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.4356</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0420</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.7093</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0171</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.8778</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0047</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.8344</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.1456</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.9053</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0221</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.7201</t>
+  </si>
+  <si>
+    <t>Best-v5-Model  09.12.2024 - 20.47</t>
+  </si>
+  <si>
+    <t>Best-v6-Model  09.12.2024 - 21.23</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.8535</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.1083</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.9419</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0188</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.9239</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.1653</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.9353</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0280</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.8795</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0994</t>
+  </si>
+  <si>
+    <t>Best-v7-Model  09.12.2024 - 22.01</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.8914</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0286</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.9349</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0022</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.9242</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.2066</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.9399</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0094</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.8831</t>
+  </si>
+  <si>
+    <t>Depression Probability: 0.0712</t>
   </si>
 </sst>
 </file>
@@ -414,173 +612,751 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A41"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="45.77734375" customWidth="1"/>
-    <col min="2" max="2" width="36.5546875" customWidth="1"/>
-    <col min="3" max="3" width="34.109375" customWidth="1"/>
-    <col min="4" max="4" width="44.44140625" customWidth="1"/>
+    <col min="1" max="1" width="27.77734375" customWidth="1"/>
+    <col min="2" max="3" width="28" customWidth="1"/>
+    <col min="4" max="4" width="28.21875" customWidth="1"/>
+    <col min="5" max="5" width="27.5546875" customWidth="1"/>
+    <col min="6" max="6" width="26.33203125" customWidth="1"/>
+    <col min="7" max="7" width="49.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>1</v>
+      </c>
+      <c r="G3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F4" t="s">
+        <v>2</v>
+      </c>
+      <c r="G4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" t="s">
+        <v>69</v>
+      </c>
+      <c r="G5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F7" t="s">
+        <v>4</v>
+      </c>
+      <c r="G7" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E8" t="s">
+        <v>5</v>
+      </c>
+      <c r="F8" t="s">
+        <v>5</v>
+      </c>
+      <c r="G8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" t="s">
+        <v>59</v>
+      </c>
+      <c r="F9" t="s">
+        <v>70</v>
+      </c>
+      <c r="G9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B12" t="s">
+        <v>2</v>
+      </c>
+      <c r="C12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F12" t="s">
+        <v>2</v>
+      </c>
+      <c r="G12" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E13" t="s">
+        <v>60</v>
+      </c>
+      <c r="F13" t="s">
+        <v>71</v>
+      </c>
+      <c r="G13" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15" t="s">
+        <v>9</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+      <c r="G15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>5</v>
+      </c>
+      <c r="E16" t="s">
+        <v>5</v>
+      </c>
+      <c r="F16" t="s">
+        <v>5</v>
+      </c>
+      <c r="G16" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" t="s">
+        <v>51</v>
+      </c>
+      <c r="E17" t="s">
+        <v>61</v>
+      </c>
+      <c r="F17" t="s">
+        <v>72</v>
+      </c>
+      <c r="G17" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B20" t="s">
+        <v>2</v>
+      </c>
+      <c r="C20" t="s">
+        <v>2</v>
+      </c>
+      <c r="D20" t="s">
+        <v>2</v>
+      </c>
+      <c r="E20" t="s">
+        <v>2</v>
+      </c>
+      <c r="F20" t="s">
+        <v>2</v>
+      </c>
+      <c r="G20" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B21" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" t="s">
+        <v>41</v>
+      </c>
+      <c r="D21" t="s">
+        <v>52</v>
+      </c>
+      <c r="E21" t="s">
+        <v>62</v>
+      </c>
+      <c r="F21" t="s">
+        <v>73</v>
+      </c>
+      <c r="G21" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B23" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" t="s">
+        <v>13</v>
+      </c>
+      <c r="E23" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B24" t="s">
+        <v>5</v>
+      </c>
+      <c r="C24" t="s">
+        <v>5</v>
+      </c>
+      <c r="D24" t="s">
+        <v>5</v>
+      </c>
+      <c r="E24" t="s">
+        <v>5</v>
+      </c>
+      <c r="F24" t="s">
+        <v>5</v>
+      </c>
+      <c r="G24" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B25" t="s">
+        <v>30</v>
+      </c>
+      <c r="C25" t="s">
+        <v>42</v>
+      </c>
+      <c r="D25" t="s">
+        <v>53</v>
+      </c>
+      <c r="E25" t="s">
+        <v>63</v>
+      </c>
+      <c r="F25" t="s">
+        <v>74</v>
+      </c>
+      <c r="G25" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B27" t="s">
+        <v>15</v>
+      </c>
+      <c r="C27" t="s">
+        <v>15</v>
+      </c>
+      <c r="D27" t="s">
+        <v>15</v>
+      </c>
+      <c r="E27" t="s">
+        <v>15</v>
+      </c>
+      <c r="F27" t="s">
+        <v>15</v>
+      </c>
+      <c r="G27" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B28" t="s">
+        <v>2</v>
+      </c>
+      <c r="C28" t="s">
+        <v>2</v>
+      </c>
+      <c r="D28" t="s">
+        <v>2</v>
+      </c>
+      <c r="E28" t="s">
+        <v>2</v>
+      </c>
+      <c r="F28" t="s">
+        <v>2</v>
+      </c>
+      <c r="G28" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B29" t="s">
+        <v>31</v>
+      </c>
+      <c r="C29" t="s">
+        <v>43</v>
+      </c>
+      <c r="D29" t="s">
+        <v>54</v>
+      </c>
+      <c r="E29" t="s">
+        <v>64</v>
+      </c>
+      <c r="F29" t="s">
+        <v>75</v>
+      </c>
+      <c r="G29" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B31" t="s">
+        <v>17</v>
+      </c>
+      <c r="C31" t="s">
+        <v>17</v>
+      </c>
+      <c r="D31" t="s">
+        <v>17</v>
+      </c>
+      <c r="E31" t="s">
+        <v>17</v>
+      </c>
+      <c r="F31" t="s">
+        <v>17</v>
+      </c>
+      <c r="G31" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B32" t="s">
+        <v>5</v>
+      </c>
+      <c r="C32" t="s">
+        <v>5</v>
+      </c>
+      <c r="D32" t="s">
+        <v>5</v>
+      </c>
+      <c r="E32" t="s">
+        <v>5</v>
+      </c>
+      <c r="F32" t="s">
+        <v>5</v>
+      </c>
+      <c r="G32" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B33" t="s">
+        <v>32</v>
+      </c>
+      <c r="C33" t="s">
+        <v>44</v>
+      </c>
+      <c r="D33" t="s">
+        <v>55</v>
+      </c>
+      <c r="E33" t="s">
+        <v>65</v>
+      </c>
+      <c r="F33" t="s">
+        <v>76</v>
+      </c>
+      <c r="G33" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B35" t="s">
+        <v>19</v>
+      </c>
+      <c r="C35" t="s">
+        <v>19</v>
+      </c>
+      <c r="D35" t="s">
+        <v>19</v>
+      </c>
+      <c r="E35" t="s">
+        <v>19</v>
+      </c>
+      <c r="F35" t="s">
+        <v>19</v>
+      </c>
+      <c r="G35" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B36" t="s">
+        <v>5</v>
+      </c>
+      <c r="C36" t="s">
+        <v>2</v>
+      </c>
+      <c r="D36" t="s">
+        <v>5</v>
+      </c>
+      <c r="E36" t="s">
+        <v>2</v>
+      </c>
+      <c r="F36" t="s">
+        <v>2</v>
+      </c>
+      <c r="G36" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B37" t="s">
+        <v>33</v>
+      </c>
+      <c r="C37" t="s">
+        <v>45</v>
+      </c>
+      <c r="D37" t="s">
+        <v>56</v>
+      </c>
+      <c r="E37" t="s">
+        <v>66</v>
+      </c>
+      <c r="F37" t="s">
+        <v>77</v>
+      </c>
+      <c r="G37" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B39" t="s">
+        <v>21</v>
+      </c>
+      <c r="C39" t="s">
+        <v>21</v>
+      </c>
+      <c r="D39" t="s">
+        <v>21</v>
+      </c>
+      <c r="E39" t="s">
+        <v>21</v>
+      </c>
+      <c r="F39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G39" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B40" t="s">
+        <v>5</v>
+      </c>
+      <c r="C40" t="s">
+        <v>5</v>
+      </c>
+      <c r="D40" t="s">
+        <v>5</v>
+      </c>
+      <c r="E40" t="s">
+        <v>5</v>
+      </c>
+      <c r="F40" t="s">
+        <v>5</v>
+      </c>
+      <c r="G40" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>22</v>
+      </c>
+      <c r="B41" t="s">
+        <v>34</v>
+      </c>
+      <c r="C41" t="s">
+        <v>46</v>
+      </c>
+      <c r="D41" t="s">
+        <v>57</v>
+      </c>
+      <c r="E41" t="s">
+        <v>36</v>
+      </c>
+      <c r="F41" t="s">
+        <v>78</v>
+      </c>
+      <c r="G41" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>